<commit_message>
fix(excel): store baseline promotion cost as numeric zero to prevent formula type mismatch
</commit_message>
<xml_diff>
--- a/excel/scenario_model/trade_promotion_scenario_model.xlsx
+++ b/excel/scenario_model/trade_promotion_scenario_model.xlsx
@@ -800,10 +800,8 @@
           <t>Total Promotion Cost (Discount + Budget)</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>₹0.00</t>
-        </is>
+      <c r="G14" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H14" s="9">
         <f>H13+C10</f>

</xml_diff>

<commit_message>
fix(excel): standardize currency format strings across generator and tests to prevent locale errors
</commit_message>
<xml_diff>
--- a/excel/scenario_model/trade_promotion_scenario_model.xlsx
+++ b/excel/scenario_model/trade_promotion_scenario_model.xlsx
@@ -16,12 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.00x"/>
-    <numFmt numFmtId="167" formatCode="#,##0 bps"/>
-    <numFmt numFmtId="168" formatCode="₹#,##0"/>
+    <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -32,37 +30,37 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F4E79"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -127,44 +125,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -562,7 +560,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Interactive B2B trade discount sensitivity &amp; net incremental gross profit model</t>
+          <t>B2B wholesale trade discount sensitivity and net incremental margin model</t>
         </is>
       </c>
     </row>
@@ -611,7 +609,7 @@
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Product List Price (₹)</t>
+          <t>Product List Price ($)</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
@@ -638,7 +636,7 @@
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Unit Cost of Goods Sold (₹)</t>
+          <t>Unit Cost of Goods Sold ($)</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
@@ -692,7 +690,7 @@
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Campaign Fixed Promotional Budget (₹)</t>
+          <t>Campaign Fixed Promotional Budget ($)</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
@@ -820,14 +818,14 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>5. SENSITIVITY TABLE: NET INCREMENTAL GROSS PROFIT (₹)</t>
+          <t>5. SENSITIVITY TABLE: NET INCREMENTAL GROSS PROFIT ($)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Net Incremental Gross Profit (₹)</t>
+          <t>Net Incremental Gross Profit ($)</t>
         </is>
       </c>
       <c r="C18" s="14">

</xml_diff>